<commit_message>
updates to cost main
</commit_message>
<xml_diff>
--- a/Launcher DB 251 redux.xlsx
+++ b/Launcher DB 251 redux.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdepaor2\Desktop\ORLA_Lander_Mission_Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D6FCE7-DDBB-46F3-AF26-6FB63778EE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089B9C7D-858E-4D4C-B63D-BB5B134EBE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{69C8745A-9C92-45EB-911F-DC35D6424AAB}"/>
+    <workbookView xWindow="585" yWindow="1170" windowWidth="23235" windowHeight="11685" xr2:uid="{69C8745A-9C92-45EB-911F-DC35D6424AAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -495,17 +495,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88A460DE-E610-40B3-9869-D6A1A40F73E6}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.33203125" customWidth="1"/>
-    <col min="6" max="8" width="15.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" customWidth="1"/>
+    <col min="6" max="8" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,7 +531,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -542,26 +542,26 @@
         <v>3300</v>
       </c>
       <c r="D2" s="5">
-        <f>B2/C2</f>
+        <f t="shared" ref="D2:D7" si="0">B2/C2</f>
         <v>11212.121212121212</v>
       </c>
       <c r="E2" s="5">
         <v>698</v>
       </c>
       <c r="F2" s="2">
-        <f>0.5*(C2+E2)*9500^2</f>
+        <f t="shared" ref="F2:F7" si="1">0.5*(C2+E2)*9500^2</f>
         <v>180409750000</v>
       </c>
       <c r="G2" s="7">
-        <f>2*F2/(13400^2)-E2</f>
+        <f t="shared" ref="G2:G7" si="2">2*F2/(13400^2)-E2</f>
         <v>1311.4648028514146</v>
       </c>
       <c r="H2" s="7">
-        <f>B2/G2</f>
+        <f t="shared" ref="H2:H7" si="3">B2/G2</f>
         <v>28212.728179630758</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -572,26 +572,26 @@
         <v>22800</v>
       </c>
       <c r="D3" s="5">
-        <f>B3/C3</f>
+        <f t="shared" si="0"/>
         <v>2938.5964912280701</v>
       </c>
       <c r="E3" s="5">
         <v>3900</v>
       </c>
       <c r="F3" s="2">
-        <f>0.5*(C3+E3)*9500^2</f>
+        <f t="shared" si="1"/>
         <v>1204837500000</v>
       </c>
       <c r="G3" s="7">
-        <f>2*F3/(13400^2)-E3</f>
+        <f t="shared" si="2"/>
         <v>9519.8875027845843</v>
       </c>
       <c r="H3" s="7">
-        <f>B3/G3</f>
+        <f t="shared" si="3"/>
         <v>7037.898292432802</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -602,26 +602,26 @@
         <v>18831</v>
       </c>
       <c r="D4" s="5">
-        <f>B4/C4</f>
+        <f t="shared" si="0"/>
         <v>3876.5864797408531</v>
       </c>
       <c r="E4" s="5">
         <v>2462</v>
       </c>
       <c r="F4" s="2">
-        <f>0.5*(C4+E4)*9500^2</f>
+        <f t="shared" si="1"/>
         <v>960846625000</v>
       </c>
       <c r="G4" s="7">
-        <f>2*F4/(13400^2)-E4</f>
+        <f t="shared" si="2"/>
         <v>8240.2346290933401</v>
       </c>
       <c r="H4" s="7">
-        <f>B4/G4</f>
+        <f t="shared" si="3"/>
         <v>8858.9710470455466</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -632,26 +632,26 @@
         <v>21650</v>
       </c>
       <c r="D5" s="3">
-        <f>B5/C5</f>
+        <f t="shared" si="0"/>
         <v>5311.778290993072</v>
       </c>
       <c r="E5" s="6">
         <v>3500</v>
       </c>
       <c r="F5" s="2">
-        <f>0.5*(C5+E5)*9500^2</f>
+        <f t="shared" si="1"/>
         <v>1134893750000</v>
       </c>
       <c r="G5" s="7">
-        <f>2*F5/(13400^2)-E5</f>
+        <f t="shared" si="2"/>
         <v>9140.8303631098242</v>
       </c>
       <c r="H5" s="7">
-        <f>B5/G5</f>
+        <f t="shared" si="3"/>
         <v>12580.913924856557</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
@@ -662,26 +662,26 @@
         <v>63800</v>
       </c>
       <c r="D6" s="3">
-        <f>B6/C6</f>
+        <f t="shared" si="0"/>
         <v>2351.0971786833857</v>
       </c>
       <c r="E6" s="3">
         <v>3900</v>
       </c>
       <c r="F6" s="2">
-        <f>0.5*(C6+E6)*9500^2</f>
+        <f t="shared" si="1"/>
         <v>3054962500000</v>
       </c>
       <c r="G6" s="7">
-        <f>2*F6/(13400^2)-E6</f>
+        <f t="shared" si="2"/>
         <v>30127.205390955671</v>
       </c>
       <c r="H6" s="7">
-        <f>B6/G6</f>
+        <f t="shared" si="3"/>
         <v>4978.8886175626067</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -692,22 +692,22 @@
         <v>95000</v>
       </c>
       <c r="D7" s="3">
-        <f>B7/C7</f>
+        <f t="shared" si="0"/>
         <v>21052.63157894737</v>
       </c>
       <c r="E7" s="3">
         <v>3490</v>
       </c>
       <c r="F7" s="2">
-        <f>0.5*(C7+E7)*9500^2</f>
+        <f t="shared" si="1"/>
         <v>4444361250000</v>
       </c>
       <c r="G7" s="7">
-        <f>2*F7/(13400^2)-E7</f>
+        <f t="shared" si="2"/>
         <v>46012.798507462685</v>
       </c>
       <c r="H7" s="7">
-        <f>B7/G7</f>
+        <f t="shared" si="3"/>
         <v>43466.167346366157</v>
       </c>
     </row>

</xml_diff>